<commit_message>
Phase 3: score_history writes, art_literature table + API + UI
</commit_message>
<xml_diff>
--- a/Design doc Atelier.xlsx
+++ b/Design doc Atelier.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10404"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/satishfactory.art/Projects/atelier/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9FAE4026-F605-FB4E-87A1-FA61DBB01058}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29F5E7ED-FC35-DA47-919F-CA6DAFFD553B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16240" activeTab="4" xr2:uid="{22BCD640-8102-4646-A614-59583DA99F09}"/>
+    <workbookView xWindow="380" yWindow="600" windowWidth="28040" windowHeight="16240" activeTab="6" xr2:uid="{22BCD640-8102-4646-A614-59583DA99F09}"/>
   </bookViews>
   <sheets>
     <sheet name="Tables" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,9 @@
     <sheet name="Vector embeddings" sheetId="2" r:id="rId3"/>
     <sheet name="Shared intelligence" sheetId="3" r:id="rId4"/>
     <sheet name="Retrieval Pipeline" sheetId="5" r:id="rId5"/>
+    <sheet name="Prompt context" sheetId="6" r:id="rId6"/>
+    <sheet name="Sheet2" sheetId="7" r:id="rId7"/>
+    <sheet name="Prompt" sheetId="8" r:id="rId8"/>
   </sheets>
   <calcPr calcId="181029"/>
   <extLst>
@@ -40,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="275" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="324">
   <si>
     <t xml:space="preserve"> Table </t>
   </si>
@@ -848,6 +851,351 @@
   </si>
   <si>
     <t>Ask for an example of a retrieval call for evaliate painting  and exact backend process mao</t>
+  </si>
+  <si>
+    <t>| callType | Fetches | DB queries |</t>
+  </si>
+  <si>
+    <t>        |----------|---------|-----------|</t>
+  </si>
+  <si>
+    <t>        | evaluate_painting | painting_history (companion_conversations last 5), allSessions (painting_sessions all), wipSessions (last 3), studio_state (studio_states), painting_subject, recent_paintings (paintings last 5), evolution_metrics, artist_cross_summary (artist_profiles), style_protocol (artist_style_protocols always) | 9 queries |</t>
+  </si>
+  <si>
+    <t>        | companion_dialogue | recent_dialogue (companion_conversations last 6), current_painting (painting_sessions latest), studio_state, painting_subject, style_protocol | 5 queries |</t>
+  </si>
+  <si>
+    <t>        | generate_blog | all_wip_sessions (painting_sessions all), painting_subject, linked_inspirations (inspirations by painting), studio_sessions (last 3), style_protocol | 5 queries |</t>
+  </si>
+  <si>
+    <t>        | morning_message | recent_paintings (last 5), open_wips (last 3), top_inspirations (top 3), evolution_metrics, artist_cross_summary, style_protocol | 6 queries |</t>
+  </si>
+  <si>
+    <t>        | analyse_session | rolling_summary (paintings), last_session_summary (painting_sessions), style_protocol | 3 queries |</t>
+  </si>
+  <si>
+    <t>        | session_dialogue | rolling_summary, session_transcript (from request body), style_protocol | 2 queries |</t>
+  </si>
+  <si>
+    <t>        | update_artist_summary | cross_painting_summaries (last 5 paintings with rolling_summary), style_protocol | 2 queries |</t>
+  </si>
+  <si>
+    <t>        | regenerate_bio | recent_paintings, top_inspirations, style_protocol | 3 queries |</t>
+  </si>
+  <si>
+    <t>        | collector_brief | rolling_summary, painting_history, painting_subject, top_inspirations, style_protocol | 5 queries |</t>
+  </si>
+  <si>
+    <t>        | wip_vision_prompt | (none — paintingImageUrl passed directly), style_protocol | 1 query |</t>
+  </si>
+  <si>
+    <t>        **Note:** `artist_style_protocols` is fetched on EVERY call regardless of callType — not gated by CALL_CONFIG.fetch. This means it runs even for `wip_vision_prompt` and `update_artist_summary` where style corrections are irrelevant.</t>
+  </si>
+  <si>
+    <t># PART 5 — PROMPT CONTEXT</t>
+  </si>
+  <si>
+    <t>## System prompt (static layer)</t>
+  </si>
+  <si>
+    <t>**Primary source:** `prompt_parameters` table (columns: component, content, component_order, active, component_type)</t>
+  </si>
+  <si>
+    <t>**Fallback:** `private/artmind_system_prompt.txt`</t>
+  </si>
+  <si>
+    <t>**Loaded:** On every API call (with Anthropic prompt caching — ephemeral cache_control)</t>
+  </si>
+  <si>
+    <t>**Content:** Companion persona, evaluation framework, scoring rubric, secret recipe</t>
+  </si>
+  <si>
+    <t>Current state: prompt_parameters table may not exist in DB → falls back to file on every call. This means the system prompt cannot be edited without touching the file and restarting the server.</t>
+  </si>
+  <si>
+    <t>## Dynamic context (per-call layer)</t>
+  </si>
+  <si>
+    <t>Injected as a second system block (NOT cached — changes every call).</t>
+  </si>
+  <si>
+    <t>Built by `buildDynamicContextString()` — see Part 4 for full structure.</t>
+  </si>
+  <si>
+    <t>## Token budget analysis (evaluate_painting)</t>
+  </si>
+  <si>
+    <t>| Component | Approx tokens |</t>
+  </si>
+  <si>
+    <t>|-----------|--------------|</t>
+  </si>
+  <si>
+    <t>| System prompt (static, cached) | ~800–1,200 |</t>
+  </si>
+  <si>
+    <t>| Dynamic context | ~300–600 |</t>
+  </si>
+  <si>
+    <t>| Image(s) — 1024px JPEG | ~800–1,600 per image |</t>
+  </si>
+  <si>
+    <t>| User message | ~20–50 |</t>
+  </si>
+  <si>
+    <t>| Max output | 1,500 |</t>
+  </si>
+  <si>
+    <t>| **Total per 1-image evaluation** | **~3,400–4,000** |</t>
+  </si>
+  <si>
+    <t>| **Total per 3-image evaluation** | **~5,800–7,000** |</t>
+  </si>
+  <si>
+    <t>- ✅ Static prompt with Anthropic prompt caching (ephemeral) — saves ~800 tokens on repeated calls</t>
+  </si>
+  <si>
+    <t>- ✅ Dynamic context string per callType — only fetches what each call needs</t>
+  </si>
+  <si>
+    <t>- ✅ Score progression with deltas (v1:72 → v2:78(+6))</t>
+  </si>
+  <si>
+    <t>- ✅ Cross-painting summary injected into evaluate + morning</t>
+  </si>
+  <si>
+    <t>- ✅ Style protocol corrections (if table exists)</t>
+  </si>
+  <si>
+    <t>- ✅ Linked inspirations in blog generation</t>
+  </si>
+  <si>
+    <t>- ✅ Image resizing before Claude API (1024px — saves 60–70% image tokens)</t>
+  </si>
+  <si>
+    <t>- ❌ Art literature / reading list in context — no table, no injection</t>
+  </si>
+  <si>
+    <t>- ❌ Masterpiece analysis in context — no table, no injection</t>
+  </si>
+  <si>
+    <t>- ❌ Companion persona as DB-editable entity — locked in file</t>
+  </si>
+  <si>
+    <t>- ❌ Semantic context retrieval — cannot retrieve "most relevant past conversation"</t>
+  </si>
+  <si>
+    <t>- ❌ painting_sessions.what_changed / what_to_do_next — fields exist in context builder but nothing populates them</t>
+  </si>
+  <si>
+    <t>- ❌ painting_subjects — UI to set artist's confirmed intention does not exist</t>
+  </si>
+  <si>
+    <t>- ❌ Prompt parameter hot-editing — table may not exist, falls back to file</t>
+  </si>
+  <si>
+    <t>## Open items — prompt context</t>
+  </si>
+  <si>
+    <t>1. System prompt cannot be updated without file edit + server restart (prompt_parameters table likely doesn't exist)</t>
+  </si>
+  <si>
+    <t>2. `what_changed` and `what_to_do_next` fields in painting_sessions are serialised into context but UI has no input for them — always null</t>
+  </si>
+  <si>
+    <t>3. No token counting or context overflow protection — if rolling_summary grows very long, context could silently degrade</t>
+  </si>
+  <si>
+    <t>4. Linked inspirations require inspirations.linked_paintings array to be populated — no UI to do this</t>
+  </si>
+  <si>
+    <t>5. `painting_subjects` table (artist's confirmed intention) has no UI entry point</t>
+  </si>
+  <si>
+    <t>---</t>
+  </si>
+  <si>
+    <t># PART 6 — DECISION QUESTIONS FOR NEXT STEPS</t>
+  </si>
+  <si>
+    <t>## On the database</t>
+  </si>
+  <si>
+    <t>**Q1.** ✅ RESOLVED 2026-04-07 — All 5 tables created via migration_missing_tables.sql. Intelligence layer now fully active.</t>
+  </si>
+  <si>
+    <t>**Q2.** `paintings` has 10+ columns that are written by Claude (viewer_experience, practice_connection, appraisal_develop, market_positioning, bot_* scores) but never displayed in any UI. Do you want to surface any of these, or are they legacy?</t>
+  </si>
+  <si>
+    <t>**Q3.** `artist_profiles` has both `practice_description` (user-editable) and `practice_statement` (AI-regenerated). Should these be unified into one field with an edit/regenerate toggle?</t>
+  </si>
+  <si>
+    <t>**Q4.** `city` and `country` columns exist separately from `location` (a single text field in the edit form). Should the form be updated to use them, or should city/country be removed?</t>
+  </si>
+  <si>
+    <t>## On vector embeddings</t>
+  </si>
+  <si>
+    <t>**Q5.** Should embeddings be generated for companion_conversations? This would enable true semantic retrieval: "find past evaluations where I discussed light." Adds ~$0.02/1M tokens cost but enables RAG.</t>
+  </si>
+  <si>
+    <t>**Q6.** Should masterpiece paintings (type='masterpiece') be included in the embedding space for similar_paintings? Currently excluded by the filter.</t>
+  </si>
+  <si>
+    <t>**Q7.** Should an ivfflat index be added to paintings.embedding now, or wait until &gt;100 paintings exist?</t>
+  </si>
+  <si>
+    <t>## On companion intelligence (I8 — new)</t>
+  </si>
+  <si>
+    <t>**Q8.** Art library — what format? A simple `art_library` table with (title, author, type, notes, userId) that the artist populates? Or should this be captured during onboarding only?</t>
+  </si>
+  <si>
+    <t>**Q9.** Masterpiece visual analysis — should Claude analyse the masterpiece images once and cache in DB (per painting, shared across users), or re-analyse per artist with their personal context injected?</t>
+  </si>
+  <si>
+    <t>**Q10.** The companion persona — do you want to give it a name and a distinct voice (e.g., a named studio assistant character)? This would be written into the system prompt and potentially configurable.</t>
+  </si>
+  <si>
+    <t>**Q11.** What's the priority order for I8 features?</t>
+  </si>
+  <si>
+    <t>- (a) Art library table + onboarding screen + context injection</t>
+  </si>
+  <si>
+    <t>- (b) Masterpiece analysis (analyse_masterpiece callType + MasterpieceDetail screen)</t>
+  </si>
+  <si>
+    <t>- (c) Companion persona DB-editable</t>
+  </si>
+  <si>
+    <t>- (d) All together in one session</t>
+  </si>
+  <si>
+    <t>## On shared intelligence</t>
+  </si>
+  <si>
+    <t>**Q12.** Should the companion reference other artists' anonymised patterns? (e.g., "80% of artists at your score range struggle with backgrounds") — this requires a shared intelligence layer across users. Worth designing?</t>
+  </si>
+  <si>
+    <t>**Q13.** Cross-painting summary currently synthesises rolling_summaries. Should it also synthesise studio_states (mood patterns over time)?</t>
+  </si>
+  <si>
+    <t>## On retrieval</t>
+  </si>
+  <si>
+    <t>**Q14.** `what_changed` and `what_to_do_next` columns in painting_sessions are in the context builder but nothing populates them. Add UI inputs to the journal note form, or remove from context builder?</t>
+  </si>
+  <si>
+    <t>**Q15.** Rolling summary has no length cap. Should it be capped (e.g., 400 words) and rewritten on each session, or kept as a growing document?</t>
+  </si>
+  <si>
+    <t>**Q16.** Linked inspirations (inspirations.linked_paintings[]) cannot be set from any current UI. Add a "link to painting" button in the influences section, or keep as manual Supabase entry?</t>
+  </si>
+  <si>
+    <t>## On deployment readiness</t>
+  </si>
+  <si>
+    <t>**Q17.** Before deploying, should the unconfirmed tables be verified and created if missing? This is a ~30-minute Supabase dashboard task.</t>
+  </si>
+  <si>
+    <t>**Q18.** ✅ RESOLVED 2026-04-07 — migration_relink_owner.sql has been run. All existing data is linked to the real Auth UUID.</t>
+  </si>
+  <si>
+    <t>## ATELIER PROJECT UPDATE — BATCH INSTRUCTIONS
+### 1. DATABASE FIXES
+- Add `user_id` FK to paintings table (link to auth.users)
+- Identify &amp; populate blank painting columns with seed data
+- Seed these empty tables with realistic test data (2-3 rows each):
+  studio_states, evolution_metrics, artist_style_protocols,
+  painting_subjects, prompt_parameters
+### 2. REMOVE MORNING MESSAGE
+- Delete all morning message logic (UI + API + context injection)
+- Remove from shared intelligence token injection
+- Remove from CALL_CONFIG
+### 3. FIX STYLE PROTOCOLS GATE
+- `artist_style_protocols` should only fetch when CALL_CONFIG.fetch = true
+- Do NOT fetch for: wip_vision_prompt, update_artist_summary
+### 4. PROFILE PAGE BUG
+- Cross-painting summary not showing — debug why "Evaluate painting 
+  complete" write is not surfacing on profile. Fix it.
+### 5. CREATE MISSING TABLES
+Create Supabase tables + RLS for:
+- art_literature (title, author, notes, user_id)
+- masterpiece_analysis (image_url, ai_analysis, embedding, user_id)
+- companion_persona (name, traits, tone — DB-driven not hardcoded)
+- onboarding_reading_list (user_id, book_title, added_at)
+### 6. CONNECT DISCONNECTED OBJECTS
+- inspirations → painting_subjects (link influence to intention)
+- score_history → evolution_metrics (start writing scores)
+- paintings.embedding → conversations (semantic retrieval)
+- studio_states → evolution_metrics (mood factors into growth)
+- artist_style_protocols → painting_subjects (style references intention)
+### 7. UPDATE PROJECT PLAN
+- Mark morning message as removed
+- Add new tables to schema doc
+- Document all new object relationships</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes </t>
+  </si>
+  <si>
+    <t>Viewer experience, market positioning, bot*scores, practice connection, In a very attractive manner. Generate data for these if it isn't there/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, unify but editable, so that artist can make changes and regenerate. </t>
+  </si>
+  <si>
+    <t>Ignore</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, but in a very token efficient way. Allow us to adjsut the intesity of this , dial up or down based on how much tokens are consumed . I </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yes, mut make them show in a different light so that they have different border, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">generate. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">make It multidimentional, on boading and also based on conversation reference. If I mention I came across this new book. Add it. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Masterpieces can be shared across users but the allow them to hide them by click of a button. BUT allow them to add their own reference artists. </t>
+  </si>
+  <si>
+    <t>Surprise me</t>
+  </si>
+  <si>
+    <t>### 8. MISSING FROM PREVIOUS INSTRUCTIONS
+# painting_sessions fields
+- `what_changed` and `what_to_do_next` exist in context builder but
+  are always null — add UI input fields to capture these per session
+# prompt_parameters table
+- Verify table exists in Supabase
+- If not, create it
+- Build simple admin UI to edit system prompt without file edit/restart
+# painting_subjects UI
+- No UI exists to set artist's confirmed intention
+- Add input/form on painting detail page to set painting_subjects
+# inspirations linking
+- inspirations.linked_paintings array never populated
+- Add UI to link inspirations to specific paintings
+# token protection
+- Add token counter to context builder
+- If rolling_summary exceeds limit (e.g. 2000 tokens), truncate oldest
+  entries and log warning
+# semantic search
+- Add embedding generation on conversation save
+- Retrieve top 3 most relevant past conversations by embedding similarity
+  and inject into context
+### PRIORITY ORDER
+1. prompt_parameters table (unblocks prompt editing)
+2. what_changed / what_to_do_next UI
+3. painting_subjects UI
+4. token protection
+5. semantic search
+6. inspirations linking</t>
   </si>
 </sst>
 </file>
@@ -1860,6 +2208,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
@@ -2349,6 +2698,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>
@@ -2675,12 +3025,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{61E8732A-FF2D-7F46-9238-5BCDB802D210}">
-  <dimension ref="A1:J62"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <sheetData>
     <row r="1" spans="1:10" x14ac:dyDescent="0.2">
@@ -2761,7 +3112,7 @@
       </c>
     </row>
     <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="6" t="s">
+      <c r="A17" s="1" t="s">
         <v>208</v>
       </c>
     </row>
@@ -2776,12 +3127,12 @@
       </c>
     </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="6" t="s">
+      <c r="A20" s="1" t="s">
         <v>209</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="6" t="s">
+      <c r="A21" s="1" t="s">
         <v>210</v>
       </c>
     </row>
@@ -2819,12 +3170,12 @@
       </c>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A29" s="6" t="s">
+      <c r="A29" s="1" t="s">
         <v>212</v>
       </c>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="6" t="s">
+      <c r="A30" s="1" t="s">
         <v>213</v>
       </c>
     </row>
@@ -2839,17 +3190,17 @@
       </c>
     </row>
     <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="6" t="s">
+      <c r="A33" s="1" t="s">
         <v>215</v>
       </c>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A34" s="6" t="s">
+      <c r="A34" s="1" t="s">
         <v>216</v>
       </c>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A35" s="6" t="s">
+      <c r="A35" s="1" t="s">
         <v>217</v>
       </c>
     </row>
@@ -2970,6 +3321,612 @@
     <row r="62" spans="1:1" x14ac:dyDescent="0.2">
       <c r="A62" s="6" t="s">
         <v>225</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="6" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="6" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" s="6" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" s="6" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" s="6" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" s="6" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A81" s="6" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="82" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A82" s="6" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="83" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A83" s="8"/>
+    </row>
+    <row r="84" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A84" s="6" t="s">
+        <v>241</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CA15E5DB-4F49-E548-9099-4205AE1094B6}">
+  <dimension ref="A1:A27"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="8"/>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="8"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="8"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="8"/>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="8"/>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="8"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="8"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="6" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="6" t="s">
+        <v>261</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C52DA196-9D2E-F24D-9D7B-6364B58D16D8}">
+  <dimension ref="A1:C80"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A2" s="6" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A3" s="6" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A4" s="6" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A5" s="6" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A6" s="6" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A7" s="6" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A8" s="6" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A9" s="8"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A10" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A11" s="6" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="12" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A12" s="6" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A13" s="6" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A14" s="6" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A15" s="6" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A16" s="6" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A17" s="6" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A18" s="8"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A19" s="6" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A20" s="6" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A21" s="6" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A22" s="6" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A23" s="6" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A24" s="6" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A25" s="8"/>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A26" s="6" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A27" s="8"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A28" s="6" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A29" s="8"/>
+    </row>
+    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A30" s="6" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A31" s="8"/>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A32" s="6" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A33" s="8"/>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A34" s="6" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A35" s="8"/>
+      <c r="B35" t="s">
+        <v>313</v>
+      </c>
+      <c r="C35" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A36" s="6" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A37" s="8"/>
+      <c r="C37" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A38" s="6" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A39" s="8"/>
+      <c r="C39" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A40" s="6" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A41" s="8"/>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A42" s="6" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A43" s="8"/>
+      <c r="C43" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="44" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A44" s="6" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="45" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A45" s="8"/>
+      <c r="C45" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="46" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A46" s="6" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A47" s="8"/>
+      <c r="C47" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="48" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A48" s="6" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="49" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A49" s="8"/>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A50" s="6" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A51" s="8"/>
+      <c r="C51" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A52" s="6" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A53" s="8"/>
+      <c r="C53" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A54" s="6" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A55" s="8"/>
+      <c r="C55" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A56" s="6" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A57" s="6" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="58" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A58" s="6" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A59" s="6" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A60" s="6" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="61" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A61" s="8"/>
+    </row>
+    <row r="62" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A62" s="6" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="63" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A63" s="8"/>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A64" s="6" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A65" s="8"/>
+    </row>
+    <row r="66" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A66" s="6" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="67" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A67" s="8"/>
+    </row>
+    <row r="68" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A68" s="6" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A69" s="8"/>
+    </row>
+    <row r="70" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A70" s="6" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="71" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A71" s="8"/>
+    </row>
+    <row r="72" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A72" s="6" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A73" s="8"/>
+    </row>
+    <row r="74" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A74" s="6" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A75" s="8"/>
+    </row>
+    <row r="76" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A76" s="6" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="77" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A77" s="8"/>
+    </row>
+    <row r="78" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A78" s="6" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="79" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A79" s="8"/>
+    </row>
+    <row r="80" spans="1:1" x14ac:dyDescent="0.2">
+      <c r="A80" s="6" t="s">
+        <v>311</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B245BB3B-E552-0C4A-B2BC-B158C723F18A}">
+  <dimension ref="B6:D6"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="2" max="2" width="130.83203125" customWidth="1"/>
+    <col min="4" max="4" width="56.1640625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="6" spans="2:4" ht="409" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="2" t="s">
+        <v>312</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>323</v>
       </c>
     </row>
   </sheetData>

</xml_diff>